<commit_message>
feat: add CLI, raw/processed/merged pipeline, drop synth-vuln-fixes
- main.py: rich CLI with synthesize/list commands; supports --lang,
  --sources, --cwe-types, --cwes, --min-cwe-count, --branches
- Stage 2 now saves per-dataset parquets to data/processed/<lang>/
  and merged deduplicated parquets to data/merged/<lang>_merged.parquet
- Remove synth-vuln-fixes extractor, test, and all notebook references
- Update 00_download_datasets, 01_*, 02_synthesis notebooks accordingly
- Rewrite README with full pipeline docs, dataset tables, CLI reference

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/stage1_java_stats.xlsx
+++ b/outputs/stage1_java_stats.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BY3"/>
+  <dimension ref="A1:CI3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -621,6 +621,16 @@
     <col width="16" customWidth="1" min="75" max="75"/>
     <col width="16" customWidth="1" min="76" max="76"/>
     <col width="16" customWidth="1" min="77" max="77"/>
+    <col width="16" customWidth="1" min="78" max="78"/>
+    <col width="16" customWidth="1" min="79" max="79"/>
+    <col width="16" customWidth="1" min="80" max="80"/>
+    <col width="16" customWidth="1" min="81" max="81"/>
+    <col width="16" customWidth="1" min="82" max="82"/>
+    <col width="16" customWidth="1" min="83" max="83"/>
+    <col width="16" customWidth="1" min="84" max="84"/>
+    <col width="16" customWidth="1" min="85" max="85"/>
+    <col width="16" customWidth="1" min="86" max="86"/>
+    <col width="16" customWidth="1" min="87" max="87"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -655,430 +665,490 @@
 Improper Neutralization of Input During Web Page Generation ('Cross-site Scripting')</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-611
+Improper Restriction of XML External Entity Reference</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-732
+Incorrect Permission Assignment for Critical Resource</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>CWE-22
 Improper Limitation of a Pathname to a Restricted Directory ('Path Traversal')</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-74
+Improper Neutralization of Special Elements in Output Used by a Downstream Component ('Injection')</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-502
+Deserialization of Untrusted Data</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-20
+Improper Input Validation</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-352
+Cross-Site Request Forgery (CSRF)</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-200
+Exposure of Sensitive Information to an Unauthorized Actor</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>CWE-89
 Improper Neutralization of Special Elements used in an SQL Command ('SQL Injection')</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-611
-Improper Restriction of XML External Entity Reference</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-74
-Improper Neutralization of Special Elements in Output Used by a Downstream Component ('Injection')</t>
-        </is>
-      </c>
-      <c r="K1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-502
-Deserialization of Untrusted Data</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>CWE-287
 Improper Authentication</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
+          <t>CWE-264
+Permissions, Privileges, and Access Controls</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>CWE-863
 Incorrect Authorization</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>CWE-310
+Cryptographic Issues</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-379
+Creation of Temporary File in Directory with Insecure Permissions</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-362
+Concurrent Execution using Shared Resource with Improper Synchronization ('Race Condition')</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-770
+Allocation of Resources Without Limits or Throttling</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-862
+Missing Authorization</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-347
+Improper Verification of Cryptographic Signature</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>CWE-94
 Improper Control of Generation of Code ('Code Injection')</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>CWE-918
 Server-Side Request Forgery (SSRF)</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-91
+XML Injection (aka Blind XPath Injection)</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-327
+Use of a Broken or Risky Cryptographic Algorithm</t>
+        </is>
+      </c>
+      <c r="AC1" s="4" t="inlineStr">
+        <is>
+          <t>CWE-361
+7PK - Time and State</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>CWE-668
 Exposure of Resource to Wrong Sphere</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-352
-Cross-Site Request Forgery (CSRF)</t>
-        </is>
-      </c>
-      <c r="R1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-862
-Missing Authorization</t>
-        </is>
-      </c>
-      <c r="S1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-770
-Allocation of Resources Without Limits or Throttling</t>
-        </is>
-      </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-755
+Improper Handling of Exceptional Conditions</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>CWE-400
 Uncontrolled Resource Consumption</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
-        <is>
-          <t>CWE-264
-Permissions, Privileges, and Access Controls</t>
-        </is>
-      </c>
-      <c r="V1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-362
-Concurrent Execution using Shared Resource with Improper Synchronization ('Race Condition')</t>
-        </is>
-      </c>
-      <c r="W1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-20
-Improper Input Validation</t>
-        </is>
-      </c>
-      <c r="X1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-755
-Improper Handling of Exceptional Conditions</t>
-        </is>
-      </c>
-      <c r="Y1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-200
-Exposure of Sensitive Information to an Unauthorized Actor</t>
-        </is>
-      </c>
-      <c r="Z1" s="3" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-326
+Inadequate Encryption Strength</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-269
+Improper Privilege Management</t>
+        </is>
+      </c>
+      <c r="AI1" s="4" t="inlineStr">
+        <is>
+          <t>CWE-19
+Data Processing Errors</t>
+        </is>
+      </c>
+      <c r="AJ1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-78
+Improper Neutralization of Special Elements used in an OS Command ('OS Command Injection')</t>
+        </is>
+      </c>
+      <c r="AK1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-190
+Integer Overflow or Wraparound</t>
+        </is>
+      </c>
+      <c r="AL1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-434
+Unrestricted Upload of File with Dangerous Type</t>
+        </is>
+      </c>
+      <c r="AM1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-346
+Origin Validation Error</t>
+        </is>
+      </c>
+      <c r="AN1" s="3" t="inlineStr">
         <is>
           <t>CWE-444
 Inconsistent Interpretation of HTTP Requests ('HTTP Request/Response Smuggling')</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-347
-Improper Verification of Cryptographic Signature</t>
-        </is>
-      </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AO1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-119
+Improper Restriction of Operations within the Bounds of a Memory Buffer</t>
+        </is>
+      </c>
+      <c r="AP1" s="4" t="inlineStr">
+        <is>
+          <t>CWE-320
+Key Management Errors</t>
+        </is>
+      </c>
+      <c r="AQ1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-759
+Use of a One-Way Hash without a Salt</t>
+        </is>
+      </c>
+      <c r="AR1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-338
+Use of Cryptographically Weak Pseudo-Random Number Generator (PRNG)</t>
+        </is>
+      </c>
+      <c r="AS1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-835
+Loop with Unreachable Exit Condition ('Infinite Loop')</t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-295
+Improper Certificate Validation</t>
+        </is>
+      </c>
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>CWE-77
 Improper Neutralization of Special Elements used in a Command ('Command Injection')</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-326
-Inadequate Encryption Strength</t>
-        </is>
-      </c>
-      <c r="AD1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-269
-Improper Privilege Management</t>
-        </is>
-      </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AV1" s="4" t="inlineStr">
+        <is>
+          <t>CWE-255
+Credentials Management Errors</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-798
+Use of Hard-coded Credentials</t>
+        </is>
+      </c>
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>CWE-522
 Insufficiently Protected Credentials</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-338
-Use of Cryptographically Weak Pseudo-Random Number Generator (PRNG)</t>
-        </is>
-      </c>
-      <c r="AG1" s="2" t="inlineStr">
+      <c r="AY1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-538
+Insertion of Sensitive Information into Externally-Accessible File or Directory</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
         <is>
           <t>CWE-290
 Authentication Bypass by Spoofing</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-835
-Loop with Unreachable Exit Condition ('Infinite Loop')</t>
-        </is>
-      </c>
-      <c r="AI1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-190
-Integer Overflow or Wraparound</t>
-        </is>
-      </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="BA1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-284
+Improper Access Control</t>
+        </is>
+      </c>
+      <c r="BB1" s="3" t="inlineStr">
         <is>
           <t>CWE-401
 Missing Release of Memory after Effective Lifetime</t>
         </is>
       </c>
-      <c r="AK1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-327
-Use of a Broken or Risky Cryptographic Algorithm</t>
-        </is>
-      </c>
-      <c r="AL1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-346
-Origin Validation Error</t>
-        </is>
-      </c>
-      <c r="AM1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-295
-Improper Certificate Validation</t>
-        </is>
-      </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="BC1" s="3" t="inlineStr">
         <is>
           <t>CWE-354
 Improper Validation of Integrity Check Value</t>
         </is>
       </c>
-      <c r="AO1" s="2" t="inlineStr">
+      <c r="BD1" s="2" t="inlineStr">
         <is>
           <t>CWE-787
 Out-of-bounds Write</t>
         </is>
       </c>
-      <c r="AP1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-732
-Incorrect Permission Assignment for Critical Resource</t>
-        </is>
-      </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="BE1" s="3" t="inlineStr">
         <is>
           <t>CWE-384
 Session Fixation</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="BF1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-428
+Unquoted Search Path or Element</t>
+        </is>
+      </c>
+      <c r="BG1" s="4" t="inlineStr">
+        <is>
+          <t>CWE-254
+7PK - Security Features</t>
+        </is>
+      </c>
+      <c r="BH1" s="3" t="inlineStr">
         <is>
           <t>CWE-1321
 Improperly Controlled Modification of Object Prototype Attributes ('Prototype Pollution')</t>
         </is>
       </c>
-      <c r="AS1" s="2" t="inlineStr">
+      <c r="BI1" s="2" t="inlineStr">
         <is>
           <t>CWE-209
 Generation of Error Message Containing Sensitive Information</t>
         </is>
       </c>
-      <c r="AT1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-434
-Unrestricted Upload of File with Dangerous Type</t>
-        </is>
-      </c>
-      <c r="AU1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-538
-Insertion of Sensitive Information into Externally-Accessible File or Directory</t>
-        </is>
-      </c>
-      <c r="AV1" s="3" t="inlineStr">
+      <c r="BJ1" s="3" t="inlineStr">
         <is>
           <t>CWE-90
 Improper Neutralization of Special Elements used in an LDAP Query ('LDAP Injection')</t>
         </is>
       </c>
-      <c r="AW1" s="2" t="inlineStr">
+      <c r="BK1" s="2" t="inlineStr">
         <is>
           <t>CWE-610
 Externally Controlled Reference to a Resource in Another Sphere</t>
         </is>
       </c>
-      <c r="AX1" s="3" t="inlineStr">
+      <c r="BL1" s="3" t="inlineStr">
         <is>
           <t>CWE-307
 Improper Restriction of Excessive Authentication Attempts</t>
         </is>
       </c>
-      <c r="AY1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-284
-Improper Access Control</t>
-        </is>
-      </c>
-      <c r="AZ1" s="3" t="inlineStr">
+      <c r="BM1" s="3" t="inlineStr">
         <is>
           <t>CWE-532
 Insertion of Sensitive Information into Log File</t>
         </is>
       </c>
-      <c r="BA1" s="2" t="inlineStr">
+      <c r="BN1" s="2" t="inlineStr">
         <is>
           <t>CWE-306
 Missing Authentication for Critical Function</t>
         </is>
       </c>
-      <c r="BB1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-78
-Improper Neutralization of Special Elements used in an OS Command ('OS Command Injection')</t>
-        </is>
-      </c>
-      <c r="BC1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-91
-XML Injection (aka Blind XPath Injection)</t>
-        </is>
-      </c>
-      <c r="BD1" s="2" t="inlineStr">
+      <c r="BO1" s="2" t="inlineStr">
         <is>
           <t>CWE-916
 Use of Password Hash With Insufficient Computational Effort</t>
         </is>
       </c>
-      <c r="BE1" s="2" t="inlineStr">
+      <c r="BP1" s="2" t="inlineStr">
         <is>
           <t>CWE-754
 Improper Check for Unusual or Exceptional Conditions</t>
         </is>
       </c>
-      <c r="BF1" s="2" t="inlineStr">
+      <c r="BQ1" s="2" t="inlineStr">
         <is>
           <t>CWE-377
 Insecure Temporary File</t>
         </is>
       </c>
-      <c r="BG1" s="2" t="inlineStr">
+      <c r="BR1" s="2" t="inlineStr">
         <is>
           <t>CWE-665
 Improper Initialization</t>
         </is>
       </c>
-      <c r="BH1" s="3" t="inlineStr">
+      <c r="BS1" s="3" t="inlineStr">
         <is>
           <t>CWE-601
 URL Redirection to Untrusted Site ('Open Redirect')</t>
         </is>
       </c>
-      <c r="BI1" s="3" t="inlineStr">
+      <c r="BT1" s="3" t="inlineStr">
         <is>
           <t>CWE-640
 Weak Password Recovery Mechanism for Forgotten Password</t>
         </is>
       </c>
-      <c r="BJ1" s="2" t="inlineStr">
+      <c r="BU1" s="2" t="inlineStr">
         <is>
           <t>CWE-116
 Improper Encoding or Escaping of Output</t>
         </is>
       </c>
-      <c r="BK1" s="3" t="inlineStr">
+      <c r="BV1" s="3" t="inlineStr">
         <is>
           <t>CWE-359
 Exposure of Private Personal Information to an Unauthorized Actor</t>
         </is>
       </c>
-      <c r="BL1" s="2" t="inlineStr">
+      <c r="BW1" s="2" t="inlineStr">
         <is>
           <t>CWE-459
 Incomplete Cleanup</t>
         </is>
       </c>
-      <c r="BM1" s="2" t="inlineStr">
+      <c r="BX1" s="2" t="inlineStr">
         <is>
           <t>CWE-312
 Cleartext Storage of Sensitive Information</t>
         </is>
       </c>
-      <c r="BN1" s="3" t="inlineStr">
+      <c r="BY1" s="3" t="inlineStr">
         <is>
           <t>CWE-274
 Improper Handling of Insufficient Privileges</t>
         </is>
       </c>
-      <c r="BO1" s="4" t="inlineStr">
-        <is>
-          <t>CWE-255
-Credentials Management Errors</t>
-        </is>
-      </c>
-      <c r="BP1" s="3" t="inlineStr">
+      <c r="BZ1" s="3" t="inlineStr">
         <is>
           <t>CWE-214
 Invocation of Process Using Visible Sensitive Information</t>
         </is>
       </c>
-      <c r="BQ1" s="2" t="inlineStr">
+      <c r="CA1" s="2" t="inlineStr">
         <is>
           <t>CWE-335
 Incorrect Usage of Seeds in Pseudo-Random Number Generator (PRNG)</t>
         </is>
       </c>
-      <c r="BR1" s="3" t="inlineStr">
+      <c r="CB1" s="3" t="inlineStr">
         <is>
           <t>CWE-476
 NULL Pointer Dereference</t>
         </is>
       </c>
-      <c r="BS1" s="2" t="inlineStr">
+      <c r="CC1" s="2" t="inlineStr">
         <is>
           <t>CWE-208
 Observable Timing Discrepancy</t>
         </is>
       </c>
-      <c r="BT1" s="2" t="inlineStr">
+      <c r="CD1" s="2" t="inlineStr">
         <is>
           <t>CWE-639
 Authorization Bypass Through User-Controlled Key</t>
         </is>
       </c>
-      <c r="BU1" s="4" t="inlineStr">
-        <is>
-          <t>CWE-310
-Cryptographic Issues</t>
-        </is>
-      </c>
-      <c r="BV1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-428
-Unquoted Search Path or Element</t>
-        </is>
-      </c>
-      <c r="BW1" s="2" t="inlineStr">
+      <c r="CE1" s="2" t="inlineStr">
         <is>
           <t>CWE-345
 Insufficient Verification of Data Authenticity</t>
         </is>
       </c>
-      <c r="BX1" s="2" t="inlineStr">
+      <c r="CF1" s="2" t="inlineStr">
         <is>
           <t>CWE-681
 Incorrect Conversion between Numeric Types</t>
         </is>
       </c>
-      <c r="BY1" s="2" t="inlineStr">
+      <c r="CG1" s="2" t="inlineStr">
         <is>
           <t>CWE-829
 Inclusion of Functionality from Untrusted Control Sphere</t>
+        </is>
+      </c>
+      <c r="CH1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-203
+Observable Discrepancy</t>
+        </is>
+      </c>
+      <c r="CI1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-915
+Improperly Controlled Modification of Dynamically-Determined Object Attributes</t>
         </is>
       </c>
     </row>
@@ -1104,13 +1174,13 @@
         <v>41</v>
       </c>
       <c r="G2" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="6" t="n">
         <v>30</v>
-      </c>
-      <c r="H2" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="I2" s="6" t="n">
-        <v>19</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>15</v>
@@ -1119,149 +1189,133 @@
         <v>15</v>
       </c>
       <c r="L2" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="N2" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="O2" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="P2" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="M2" s="6" t="n">
+      <c r="Q2" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="R2" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="N2" s="6" t="n">
+      <c r="S2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="T2" s="6" t="n"/>
+      <c r="U2" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="V2" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="W2" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="X2" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="Y2" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="O2" s="6" t="n">
+      <c r="Z2" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="P2" s="6" t="n">
+      <c r="AA2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="AC2" s="6" t="n"/>
+      <c r="AD2" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="Q2" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="R2" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="S2" s="6" t="n">
+      <c r="AE2" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AF2" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="T2" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="U2" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="V2" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="W2" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="X2" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y2" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="Z2" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA2" s="6" t="n">
+      <c r="AG2" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AB2" s="6" t="n">
+      <c r="AH2" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AC2" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AD2" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="AE2" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AF2" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG2" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH2" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="AI2" s="6" t="n">
-        <v>2</v>
-      </c>
+      <c r="AI2" s="6" t="n"/>
       <c r="AJ2" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AK2" s="6" t="n">
         <v>2</v>
       </c>
       <c r="AL2" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM2" s="6" t="n">
         <v>2</v>
       </c>
       <c r="AN2" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="AO2" s="6" t="n"/>
+      <c r="AP2" s="6" t="n"/>
+      <c r="AQ2" s="6" t="n"/>
+      <c r="AR2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AO2" s="6" t="n">
+      <c r="AS2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AP2" s="6" t="n">
+      <c r="AT2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AQ2" s="6" t="n">
+      <c r="AU2" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW2" s="6" t="n"/>
+      <c r="AX2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AR2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AX2" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="AY2" s="6" t="n">
         <v>1</v>
       </c>
       <c r="AZ2" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BA2" s="6" t="n">
         <v>1</v>
       </c>
       <c r="BB2" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BC2" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BD2" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BE2" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BF2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="BG2" s="6" t="n">
-        <v>1</v>
-      </c>
+      <c r="BG2" s="6" t="n"/>
       <c r="BH2" s="6" t="n">
         <v>1</v>
       </c>
@@ -1316,6 +1370,32 @@
       <c r="BY2" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="BZ2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CB2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CC2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CD2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CE2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CF2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CG2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH2" s="6" t="n"/>
+      <c r="CI2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -1324,71 +1404,161 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>489</v>
+        <v>1126</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>0</v>
+        <v>563</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>489</v>
+        <v>563</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="8" t="n"/>
-      <c r="J3" s="8" t="n"/>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="8" t="n"/>
-      <c r="M3" s="8" t="n"/>
-      <c r="N3" s="8" t="n"/>
-      <c r="O3" s="8" t="n"/>
-      <c r="P3" s="8" t="n"/>
-      <c r="Q3" s="8" t="n"/>
-      <c r="R3" s="8" t="n"/>
-      <c r="S3" s="8" t="n"/>
-      <c r="T3" s="8" t="n"/>
-      <c r="U3" s="8" t="n"/>
-      <c r="V3" s="8" t="n"/>
-      <c r="W3" s="8" t="n"/>
-      <c r="X3" s="8" t="n"/>
-      <c r="Y3" s="8" t="n"/>
-      <c r="Z3" s="8" t="n"/>
-      <c r="AA3" s="8" t="n"/>
-      <c r="AB3" s="8" t="n"/>
-      <c r="AC3" s="8" t="n"/>
+        <v>47</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="P3" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q3" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="R3" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="S3" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="T3" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="U3" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="V3" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="W3" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="X3" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AA3" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="AB3" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="AC3" s="8" t="n">
+        <v>10</v>
+      </c>
       <c r="AD3" s="8" t="n"/>
-      <c r="AE3" s="8" t="n"/>
+      <c r="AE3" s="8" t="n">
+        <v>5</v>
+      </c>
       <c r="AF3" s="8" t="n"/>
-      <c r="AG3" s="8" t="n"/>
-      <c r="AH3" s="8" t="n"/>
-      <c r="AI3" s="8" t="n"/>
-      <c r="AJ3" s="8" t="n"/>
-      <c r="AK3" s="8" t="n"/>
-      <c r="AL3" s="8" t="n"/>
-      <c r="AM3" s="8" t="n"/>
-      <c r="AN3" s="8" t="n"/>
-      <c r="AO3" s="8" t="n"/>
-      <c r="AP3" s="8" t="n"/>
-      <c r="AQ3" s="8" t="n"/>
-      <c r="AR3" s="8" t="n"/>
-      <c r="AS3" s="8" t="n"/>
-      <c r="AT3" s="8" t="n"/>
+      <c r="AG3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AH3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AI3" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="AJ3" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="AM3" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="AN3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO3" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AP3" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AQ3" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT3" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="AU3" s="8" t="n"/>
-      <c r="AV3" s="8" t="n"/>
-      <c r="AW3" s="8" t="n"/>
+      <c r="AV3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW3" s="8" t="n">
+        <v>3</v>
+      </c>
       <c r="AX3" s="8" t="n"/>
-      <c r="AY3" s="8" t="n"/>
+      <c r="AY3" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="AZ3" s="8" t="n"/>
-      <c r="BA3" s="8" t="n"/>
+      <c r="BA3" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="BB3" s="8" t="n"/>
       <c r="BC3" s="8" t="n"/>
       <c r="BD3" s="8" t="n"/>
       <c r="BE3" s="8" t="n"/>
-      <c r="BF3" s="8" t="n"/>
-      <c r="BG3" s="8" t="n"/>
+      <c r="BF3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG3" s="8" t="n">
+        <v>2</v>
+      </c>
       <c r="BH3" s="8" t="n"/>
       <c r="BI3" s="8" t="n"/>
       <c r="BJ3" s="8" t="n"/>
@@ -1407,6 +1577,20 @@
       <c r="BW3" s="8" t="n"/>
       <c r="BX3" s="8" t="n"/>
       <c r="BY3" s="8" t="n"/>
+      <c r="BZ3" s="8" t="n"/>
+      <c r="CA3" s="8" t="n"/>
+      <c r="CB3" s="8" t="n"/>
+      <c r="CC3" s="8" t="n"/>
+      <c r="CD3" s="8" t="n"/>
+      <c r="CE3" s="8" t="n"/>
+      <c r="CF3" s="8" t="n"/>
+      <c r="CG3" s="8" t="n"/>
+      <c r="CH3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="CI3" s="8" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1419,7 +1603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS3"/>
+  <dimension ref="A1:AZ3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1467,6 +1651,13 @@
     <col width="16" customWidth="1" min="43" max="43"/>
     <col width="16" customWidth="1" min="44" max="44"/>
     <col width="16" customWidth="1" min="45" max="45"/>
+    <col width="16" customWidth="1" min="46" max="46"/>
+    <col width="16" customWidth="1" min="47" max="47"/>
+    <col width="16" customWidth="1" min="48" max="48"/>
+    <col width="16" customWidth="1" min="49" max="49"/>
+    <col width="16" customWidth="1" min="50" max="50"/>
+    <col width="16" customWidth="1" min="51" max="51"/>
+    <col width="16" customWidth="1" min="52" max="52"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -1497,239 +1688,281 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
+          <t>CWE-89
+Improper Neutralization of Special Elements used in an SQL Command ('SQL Injection')</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-79
+Improper Neutralization of Input During Web Page Generation ('Cross-site Scripting')</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-330
+Use of Insufficiently Random Values</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-78
+Improper Neutralization of Special Elements used in an OS Command ('OS Command Injection')</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-22
+Improper Limitation of a Pathname to a Restricted Directory ('Path Traversal')</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-327
+Use of a Broken or Risky Cryptographic Algorithm</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>CWE-328
+Use of Weak Hash</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
           <t>CWE-190
 Integer Overflow or Wraparound</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>CWE-191
 Integer Underflow (Wrap or Wraparound)</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-501
+Trust Boundary Violation</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>CWE-129
 Improper Validation of Array Index</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>CWE-89
-Improper Neutralization of Special Elements used in an SQL Command ('SQL Injection')</t>
-        </is>
-      </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>CWE-369
 Divide By Zero</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>CWE-789
 Memory Allocation with Excessive Size Value</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>CWE-400
 Uncontrolled Resource Consumption</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-90
+Improper Neutralization of Special Elements used in an LDAP Query ('LDAP Injection')</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>CWE-113
 Improper Neutralization of CRLF Sequences in HTTP Headers ('HTTP Request/Response Splitting')</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-614
+Sensitive Cookie in HTTPS Session Without 'Secure' Attribute</t>
+        </is>
+      </c>
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>CWE-197
 Numeric Truncation Error</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>CWE-643
+Improper Neutralization of Data within XPath Expressions ('XPath Injection')</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>CWE-134
 Use of Externally-Controlled Format String</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Z1" s="3" t="inlineStr">
         <is>
           <t>CWE-80
 Improper Neutralization of Script-Related HTML Tags in a Web Page (Basic XSS)</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-643
-Improper Neutralization of Data within XPath Expressions ('XPath Injection')</t>
-        </is>
-      </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="AA1" s="3" t="inlineStr">
         <is>
           <t>CWE-15
 External Control of System or Configuration Setting</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>CWE-23
 Relative Path Traversal</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-90
-Improper Neutralization of Special Elements used in an LDAP Query ('LDAP Injection')</t>
-        </is>
-      </c>
-      <c r="U1" s="3" t="inlineStr">
+      <c r="AC1" s="3" t="inlineStr">
         <is>
           <t>CWE-470
 Use of Externally-Controlled Input to Select Classes or Code ('Unsafe Reflection')</t>
         </is>
       </c>
-      <c r="V1" s="3" t="inlineStr">
+      <c r="AD1" s="3" t="inlineStr">
         <is>
           <t>CWE-563
 Assignment to Variable without Use</t>
         </is>
       </c>
-      <c r="W1" s="3" t="inlineStr">
-        <is>
-          <t>CWE-78
-Improper Neutralization of Special Elements used in an OS Command ('OS Command Injection')</t>
-        </is>
-      </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>CWE-36
 Absolute Path Traversal</t>
         </is>
       </c>
-      <c r="Y1" s="3" t="inlineStr">
+      <c r="AF1" s="3" t="inlineStr">
         <is>
           <t>CWE-606
 Unchecked Input for Loop Condition</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>CWE-319
 Cleartext Transmission of Sensitive Information</t>
         </is>
       </c>
-      <c r="AA1" s="3" t="inlineStr">
+      <c r="AH1" s="3" t="inlineStr">
         <is>
           <t>CWE-81
 Improper Neutralization of Script in an Error Message Web Page</t>
         </is>
       </c>
-      <c r="AB1" s="3" t="inlineStr">
+      <c r="AI1" s="3" t="inlineStr">
         <is>
           <t>CWE-601
 URL Redirection to Untrusted Site ('Open Redirect')</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>CWE-83
 Improper Neutralization of Script in Attributes in a Web Page</t>
         </is>
       </c>
-      <c r="AD1" s="3" t="inlineStr">
+      <c r="AK1" s="3" t="inlineStr">
         <is>
           <t>CWE-690
 Unchecked Return Value to NULL Pointer Dereference</t>
         </is>
       </c>
-      <c r="AE1" s="3" t="inlineStr">
+      <c r="AL1" s="3" t="inlineStr">
         <is>
           <t>CWE-476
 NULL Pointer Dereference</t>
         </is>
       </c>
-      <c r="AF1" s="3" t="inlineStr">
+      <c r="AM1" s="3" t="inlineStr">
         <is>
           <t>CWE-259
 Use of Hard-coded Password</t>
         </is>
       </c>
-      <c r="AG1" s="3" t="inlineStr">
+      <c r="AN1" s="3" t="inlineStr">
         <is>
           <t>CWE-568
 finalize() Method Without super.finalize()</t>
         </is>
       </c>
-      <c r="AH1" s="3" t="inlineStr">
+      <c r="AO1" s="3" t="inlineStr">
         <is>
           <t>CWE-581
 Object Model Violation: Just One of Equals and Hashcode Defined</t>
         </is>
       </c>
-      <c r="AI1" s="3" t="inlineStr">
+      <c r="AP1" s="3" t="inlineStr">
         <is>
           <t>CWE-499
 Serializable Class Containing Sensitive Data</t>
         </is>
       </c>
-      <c r="AJ1" s="3" t="inlineStr">
+      <c r="AQ1" s="3" t="inlineStr">
         <is>
           <t>CWE-491
 Public cloneable() Method Without Final ('Object Hijack')</t>
         </is>
       </c>
-      <c r="AK1" s="3" t="inlineStr">
+      <c r="AR1" s="3" t="inlineStr">
         <is>
           <t>CWE-500
 Public Static Field Not Marked Final</t>
         </is>
       </c>
-      <c r="AL1" s="3" t="inlineStr">
+      <c r="AS1" s="3" t="inlineStr">
         <is>
           <t>CWE-561
 Dead Code</t>
         </is>
       </c>
-      <c r="AM1" s="3" t="inlineStr">
+      <c r="AT1" s="3" t="inlineStr">
         <is>
           <t>CWE-580
 clone() Method Without super.clone()</t>
         </is>
       </c>
-      <c r="AN1" s="3" t="inlineStr">
+      <c r="AU1" s="3" t="inlineStr">
         <is>
           <t>CWE-607
 Public Static Final Field References Mutable Object</t>
         </is>
       </c>
-      <c r="AO1" s="3" t="inlineStr">
+      <c r="AV1" s="3" t="inlineStr">
         <is>
           <t>CWE-582
 Array Declared Public, Final, and Static</t>
         </is>
       </c>
-      <c r="AP1" s="3" t="inlineStr">
+      <c r="AW1" s="3" t="inlineStr">
         <is>
           <t>CWE-321
 Use of Hard-coded Cryptographic Key</t>
         </is>
       </c>
-      <c r="AQ1" s="3" t="inlineStr">
+      <c r="AX1" s="3" t="inlineStr">
         <is>
           <t>CWE-256
 Plaintext Storage of a Password</t>
         </is>
       </c>
-      <c r="AR1" s="3" t="inlineStr">
+      <c r="AY1" s="3" t="inlineStr">
         <is>
           <t>CWE-315
 Cleartext Storage of Sensitive Information in a Cookie</t>
         </is>
       </c>
-      <c r="AS1" s="3" t="inlineStr">
+      <c r="AZ1" s="3" t="inlineStr">
         <is>
           <t>CWE-566
 Authorization Bypass Through User-Controlled SQL Primary Key</t>
@@ -1755,113 +1988,99 @@
         <v>40</v>
       </c>
       <c r="F2" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n">
         <v>115</v>
       </c>
-      <c r="G2" s="6" t="n">
+      <c r="N2" s="6" t="n">
         <v>92</v>
       </c>
-      <c r="H2" s="6" t="n">
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="I2" s="6" t="n">
-        <v>60</v>
-      </c>
-      <c r="J2" s="6" t="n">
+      <c r="Q2" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="K2" s="6" t="n">
+      <c r="R2" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="L2" s="6" t="n">
+      <c r="S2" s="6" t="n">
         <v>39</v>
-      </c>
-      <c r="M2" s="6" t="n">
-        <v>36</v>
-      </c>
-      <c r="N2" s="6" t="n">
-        <v>33</v>
-      </c>
-      <c r="O2" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="P2" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q2" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="R2" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="S2" s="6" t="n">
-        <v>12</v>
       </c>
       <c r="T2" s="6" t="n">
         <v>12</v>
       </c>
       <c r="U2" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="V2" s="6" t="n">
-        <v>12</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="V2" s="6" t="n"/>
       <c r="W2" s="6" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="X2" s="6" t="n">
         <v>12</v>
       </c>
       <c r="Y2" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="Z2" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="AA2" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="Z2" s="6" t="n">
+      <c r="AB2" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="AC2" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="AD2" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="AE2" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="AF2" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="AG2" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="AA2" s="6" t="n">
+      <c r="AH2" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="AB2" s="6" t="n">
+      <c r="AI2" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="AC2" s="6" t="n">
+      <c r="AJ2" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="AD2" s="6" t="n">
+      <c r="AK2" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="AE2" s="6" t="n">
+      <c r="AL2" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="AF2" s="6" t="n">
+      <c r="AM2" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="AG2" s="6" t="n">
+      <c r="AN2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AH2" s="6" t="n">
+      <c r="AO2" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="AI2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AO2" s="6" t="n">
-        <v>1</v>
-      </c>
       <c r="AP2" s="6" t="n">
         <v>1</v>
       </c>
@@ -1872,6 +2091,27 @@
         <v>1</v>
       </c>
       <c r="AS2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AW2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AY2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ2" s="6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1885,33 +2125,55 @@
         <v>2740</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>0</v>
+        <v>1415</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>2740</v>
+        <v>1325</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="8" t="n"/>
-      <c r="G3" s="8" t="n"/>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="8" t="n"/>
-      <c r="J3" s="8" t="n"/>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="8" t="n"/>
+        <v>11</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>272</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>246</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>218</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>126</v>
+      </c>
+      <c r="J3" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>130</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>129</v>
+      </c>
       <c r="M3" s="8" t="n"/>
       <c r="N3" s="8" t="n"/>
-      <c r="O3" s="8" t="n"/>
+      <c r="O3" s="8" t="n">
+        <v>83</v>
+      </c>
       <c r="P3" s="8" t="n"/>
       <c r="Q3" s="8" t="n"/>
       <c r="R3" s="8" t="n"/>
       <c r="S3" s="8" t="n"/>
-      <c r="T3" s="8" t="n"/>
+      <c r="T3" s="8" t="n">
+        <v>27</v>
+      </c>
       <c r="U3" s="8" t="n"/>
-      <c r="V3" s="8" t="n"/>
+      <c r="V3" s="8" t="n">
+        <v>36</v>
+      </c>
       <c r="W3" s="8" t="n"/>
-      <c r="X3" s="8" t="n"/>
+      <c r="X3" s="8" t="n">
+        <v>15</v>
+      </c>
       <c r="Y3" s="8" t="n"/>
       <c r="Z3" s="8" t="n"/>
       <c r="AA3" s="8" t="n"/>
@@ -1933,6 +2195,13 @@
       <c r="AQ3" s="8" t="n"/>
       <c r="AR3" s="8" t="n"/>
       <c r="AS3" s="8" t="n"/>
+      <c r="AT3" s="8" t="n"/>
+      <c r="AU3" s="8" t="n"/>
+      <c r="AV3" s="8" t="n"/>
+      <c r="AW3" s="8" t="n"/>
+      <c r="AX3" s="8" t="n"/>
+      <c r="AY3" s="8" t="n"/>
+      <c r="AZ3" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7172,7 +7441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7301,7 +7570,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>CWE-Bench-Java</t>
+          <t>CrossVul(Java)</t>
         </is>
       </c>
       <c r="B3" s="11" t="inlineStr">
@@ -7316,27 +7585,27 @@
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>GitHub iris-sast/cwe-bench-java (methods fetched from GitHub raw)</t>
+          <t>Zenodo crossvul.zip</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>vulnerable method (buggy commit)</t>
+          <t>bad_* files (vulnerable functions)</t>
         </is>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
-          <t>fixed method (fix commit)</t>
+          <t>good_* files (fixed functions)</t>
         </is>
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>project_info.csv cwe_id column</t>
+          <t>CWE-NNN directory name</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr">
         <is>
-          <t>code non-empty, CWE non-empty, method lines valid</t>
+          <t>java/ folder filter</t>
         </is>
       </c>
       <c r="I3" s="11" t="inlineStr">
@@ -7346,24 +7615,20 @@
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>4/5</t>
-        </is>
-      </c>
-      <c r="K3" s="11" t="inlineStr">
-        <is>
-          <t>methods extracted from GitHub raw API; 4 main CWEs: CWE-22, 78, 79, 94</t>
-        </is>
-      </c>
+          <t>3/5</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>CrossVul(Java)</t>
+          <t>Juliet(Java)</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>real</t>
+          <t>synth</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
@@ -7373,49 +7638,49 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>HuggingFace hitoshura25/crossvul</t>
+          <t>NIST SARD juliet-test-suite-for-java.zip</t>
         </is>
       </c>
       <c r="E4" s="10" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>*_bad.java files</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>fixed_code (fix-paired safe)</t>
+          <t>*_good*.java files</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>cwe_id column</t>
+          <t>directory name (CWE-NNN prefix)</t>
         </is>
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
-          <t>language==Java, NVD placeholder drop</t>
+          <t>filename pattern</t>
         </is>
       </c>
       <c r="I4" s="10" t="inlineStr">
         <is>
-          <t>fix-paired</t>
+          <t>pure</t>
         </is>
       </c>
       <c r="J4" s="10" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>safe only</t>
+          <t>whole .java file treated as sample</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Juliet(Java)</t>
+          <t>OWASP(Java)</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -7430,27 +7695,27 @@
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>NIST SARD juliet-test-suite-for-java.zip</t>
+          <t>OWASP GitHub BenchmarkJava</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>*_bad.java files</t>
+          <t>real vulnerability=true in expectedresults-1.2.csv</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>*_good*.java files</t>
+          <t>real vulnerability=false</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>directory name (CWE-NNN prefix)</t>
+          <t>cwe column (bare digit, normalised to CWE-NNN)</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>filename pattern</t>
+          <t>CSV join on filename (case-insensitive stem match)</t>
         </is>
       </c>
       <c r="I5" s="11" t="inlineStr">
@@ -7463,21 +7728,17 @@
           <t>5/5</t>
         </is>
       </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>whole .java file treated as sample</t>
-        </is>
-      </c>
+      <c r="K5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>OWASP(Java)</t>
+          <t>CAPEC_LLM(Java)</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>synth</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -7487,93 +7748,40 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>OWASP GitHub</t>
+          <t>GitHub llmForCapec/CAPECDatasetsLLM</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>real vulnerability=1 in expectedresults CSV</t>
+          <t>code_snippet detected as Java, CWE from description</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
-          <t>real vulnerability=0</t>
+          <t>none</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>cwe column in expectedresults CSV</t>
+          <t>CWE-NNN regex on description field</t>
         </is>
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>CSV join on filename</t>
+          <t>language detection (Java keywords), CWE regex match</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>pure</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J6" s="10" t="inlineStr">
         <is>
-          <t>5/5</t>
-        </is>
-      </c>
-      <c r="K6" s="10" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>CAPEC_LLM(Java)</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>ai</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>Java</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>GitHub llmForCapec/CAPECDatasetsLLM</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>code_snippet detected as Java, CWE from description</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>CWE-NNN regex on description field</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>language detection (Java keywords), CWE regex match</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
           <t>2/5</t>
         </is>
       </c>
-      <c r="K7" s="11" t="inlineStr">
+      <c r="K6" s="10" t="inlineStr">
         <is>
           <t>LLM-generated; CWE from CAPEC description, not per-sample</t>
         </is>

</xml_diff>